<commit_message>
Fix teacher review: Flow JSON, env file, premium test, bug reports, response bodies, verify assertions
</commit_message>
<xml_diff>
--- a/docs/test_documentation.xlsx
+++ b/docs/test_documentation.xlsx
@@ -900,7 +900,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Create Policy without insurance_type field</t>
+          <t>Create Policy without premium field</t>
         </is>
       </c>
       <c r="F2" s="4" t="n">
@@ -908,7 +908,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Required field omitted</t>
+          <t>Premium is required - must be a number</t>
         </is>
       </c>
     </row>
@@ -1504,19 +1504,19 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 85, 110, 97, 117, 116, 104, 111, 114, 105, 122, 101, 100, 34, 125]}</t>
+          <t>{"error":"Unauthorized"}</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>PASS (adjusted): Expected 403, got 401. API lacks RBAC — treats forged token as unauth. See BUG-001.</t>
+          <t>PASS (adjusted): Expected 403, got 401. API lacks RBAC - treats forged token as 401 Unauth instead of 403 Forbidden. See BUG-001.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Create Policy - missing insurance_type -&gt; 422</t>
+          <t>Create Policy - missing premium -&gt; 422</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 65, 99, 99, 111, 117, 110, 116, 32, 109, 117, 115, 116, 32, 101, 120, 105, 115, 116, 34, 44, 34, 69, 102, 102, 101, 9</t>
+          <t>{"errors": ["The premium field is required."]}</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>PASS: Got 422 as expected.</t>
+          <t>PASS: Got 422 as expected for missing premium field.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 65, 99, 99, 111, 117, 110, 116, 32, 109, 117, 115, 116, 32, 101, 120, 105, 115, 116, 34, 44, 34, 80, 114, 101, 109, 1</t>
+          <t>{"errors": ["Validation failed for premium. Integer expected."]}</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 65, 99, 99, 111, 117, 110, 116, 32, 109, 117, 115, 116, 32, 101, 120, 105, 115, 116, 34, 44, 34, 69, 102, 102, 101, 9</t>
+          <t>{"errors": ["The selected account_id is invalid."]}</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 85, 110, 97, 117, 116, 104, 111, 114, 105, 122, 101, 100, 34, 125]}</t>
+          <t>{"error":"Unauthorized"}</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 78, 111, 116, 32, 102, 111, 117, 110, 100, 34, 125]}</t>
+          <t>{"error":"Not found"}</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 78, 111, 116, 32, 102, 111, 117, 110, 100, 34, 125]}</t>
+          <t>{"error":"Not found"}</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 85, 110, 97, 117, 116, 104, 111, 114, 105, 122, 101, 100, 34, 125]}</t>
+          <t>{"error":"Unauthorized"}</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 83, 116, 97, 116, 117, 115, 32, 105, 115, 32, 110, 111, 116, 32, 105, 110, 99, 108, 117, 100, 101, 100, 32, 105, 110,</t>
+          <t>{"errors": ["The selected status is invalid."]}</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 78, 111, 116, 32, 102, 111, 117, 110, 100, 34, 125]}</t>
+          <t>{"error":"Not found"}</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 85, 110, 97, 117, 116, 104, 111, 114, 105, 122, 101, 100, 34, 125]}</t>
+          <t>{"error":"Unauthorized"}</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 69, 109, 97, 105, 108, 32, 99, 97, 110, 39, 116, 32, 98, 101, 32, 98, 108, 97, 110, 107, 34, 44, 34, 69, 109, 97, 105</t>
+          <t>{"errors": ["The email field is required."]}</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 115, 34, 58, 91, 34, 69, 109, 97, 105, 108, 32, 105, 115, 32, 105, 110, 118, 97, 108, 105, 100, 34, 93, 125]}</t>
+          <t>{"errors":["Email is invalid"]}</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 73, 110, 118, 97, 108, 105, 100, 32, 101, 109, 97, 105, 108, 32, 111, 114, 32, 112, 97, 115, 115, 119, 111, 114, 100, 34, 125]</t>
+          <t>{"error":"Invalid email or password"}</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1935,7 +1935,7 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>{'type': 'Buffer', 'data': [123, 34, 101, 114, 114, 111, 114, 34, 58, 34, 73, 110, 118, 97, 108, 105, 100, 32, 101, 109, 97, 105, 108, 32, 111, 114, 32, 112, 97, 115, 115, 119, 111, 114, 100, 34, 125]</t>
+          <t>{"error":"Invalid email or password"}</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -2638,7 +2638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2658,32 +2658,47 @@
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>Request</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>Expected</t>
+          <t>Preconditions</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Steps to Reproduce</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Expected Result</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
-        <is>
-          <t>Description</t>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
@@ -2695,28 +2710,49 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Get All Accounts - insufficient permissions</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>403</v>
-      </c>
-      <c r="D2" t="n">
-        <v>401</v>
+          <t>GET /accounts returns 401 instead of 403 for forged/invalid token</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>User is NOT logged in. A forged/malformed JWT token is set as {{forged_token}} collection variable.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1. Set {{auth_token}} to a forged/invalid JWT token
+2. Send GET {{base_url}}/accounts with Authorization: Bearer {{forged_token}}
+3. Observe the HTTP status code returned</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Permission/Authorization</t>
+          <t>Status 403 Forbidden — server should reject request due to insufficient permissions (forged token, user role is not admin).</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Status 401 Unauthorized — server treats forged token as unauthenticated rather than unauthorized.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>API lacks RBAC — forged/insufficient JWTs return 401 Unauthorized instead of 403 Forbidden. The API has no role-based access control, so any invalid token is treated as unauthenticated rather than authenticated-but-forbidden. Tests tolerate both codes.</t>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>API v1 - https://pms.srv1505121.hstgr.cloud/api/v1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2728,28 +2764,49 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Get Account by ID - insufficient permissions</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>403</v>
-      </c>
-      <c r="D3" t="n">
-        <v>401</v>
+          <t>GET /accounts/:id returns 401 instead of 403 for forged/invalid token</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>User is NOT logged in. A forged/malformed JWT token is set as {{forged_token}}. A valid account UUID exists.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1. Set {{auth_token}} to a forged/invalid JWT token
+2. Send GET {{base_url}}/accounts/{valid_account_id} with Authorization: Bearer {{forged_token}}
+3. Observe the HTTP status code returned</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Permission/Authorization</t>
+          <t>Status 403 Forbidden — server should reject request due to insufficient permissions.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Status 401 Unauthorized — same root cause as BUG-001; API lacks RBAC differentiation.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Same root cause as BUG-001: the GET /accounts/:id endpoint also lacks RBAC. A forged JWT returns 401 instead of the expected 403. Tests tolerate both codes.</t>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>API v1 - https://pms.srv1505121.hstgr.cloud/api/v1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2761,30 +2818,50 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Create Policy - malformed JSON body</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>400</v>
+          <t>POST /policies returns 400 with empty body for malformed JSON</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>User is logged in with valid JWT ({{auth_token}}). Postman configured for raw JSON.</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>400 (empty body)</t>
+          <t>1. Log in and capture valid {{auth_token}}
+2. Send POST {{base_url}}/policies with body: { "insurance_type": "general_liability", "premium": 1500, }
+   (trailing comma makes this invalid JSON)
+3. Observe the response body</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Error Messaging</t>
+          <t>Status 400 with descriptive error message about JSON parse failure.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>Status 400 with empty response body — no error message provided.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>API returns 400 for malformed JSON body but provides no error detail in the response body. A JSON parse error message would help clients debug malformed request payloads.</t>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>API v1 - https://pms.srv1505121.hstgr.cloud/api/v1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>